<commit_message>
feat: add level select panel and Mode2 MetaShell/Formation wiring
Wire LevelSelectPanel into MetaShell, refresh Formation editors/prefabs, and sync Mode2 class config with SPEC.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
@@ -172,7 +172,7 @@
     <t>1</t>
   </si>
   <si>
-    <t>App_90</t>
+    <t>App_02</t>
   </si>
   <si>
     <t>Class_Archer</t>
@@ -193,7 +193,7 @@
     <t>6</t>
   </si>
   <si>
-    <t>App_91</t>
+    <t>App_03</t>
   </si>
   <si>
     <t>Class_Mage</t>
@@ -223,7 +223,7 @@
     <t>骑士</t>
   </si>
   <si>
-    <t>App_93</t>
+    <t>App_05</t>
   </si>
   <si>
     <t>Class_Rogue</t>
@@ -238,7 +238,7 @@
     <t>5</t>
   </si>
   <si>
-    <t>App_94</t>
+    <t>App_07</t>
   </si>
   <si>
     <t>Class_Priest</t>
@@ -256,7 +256,7 @@
     <t>10</t>
   </si>
   <si>
-    <t>App_95</t>
+    <t>App_09</t>
   </si>
   <si>
     <t>Class_Berserker</t>
@@ -268,7 +268,7 @@
     <t>4</t>
   </si>
   <si>
-    <t>App_96</t>
+    <t>App_04</t>
   </si>
   <si>
     <t>Class_Ranger</t>
@@ -286,9 +286,6 @@
     <t>7</t>
   </si>
   <si>
-    <t>App_97</t>
-  </si>
-  <si>
     <t>Class_Warlock</t>
   </si>
   <si>
@@ -304,7 +301,7 @@
     <t>9</t>
   </si>
   <si>
-    <t>App_98</t>
+    <t>App_08</t>
   </si>
   <si>
     <t>Class_Paladin</t>
@@ -314,6 +311,9 @@
   </si>
   <si>
     <t>1.5</t>
+  </si>
+  <si>
+    <t>App_06</t>
   </si>
   <si>
     <t>Class_Servants</t>
@@ -341,7 +341,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -351,13 +351,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -811,153 +804,154 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -1532,7 +1526,7 @@
       <c r="K6" t="s">
         <v>59</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="L6" s="2" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1723,15 +1717,15 @@
         <v>83</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>84</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" ht="14.25" spans="1:12">
       <c r="A12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" t="s">
         <v>85</v>
-      </c>
-      <c r="B12" t="s">
-        <v>86</v>
       </c>
       <c r="C12" t="s">
         <v>56</v>
@@ -1740,13 +1734,13 @@
         <v>39</v>
       </c>
       <c r="E12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F12" t="s">
         <v>41</v>
       </c>
       <c r="G12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H12" t="s">
         <v>45</v>
@@ -1758,18 +1752,18 @@
         <v>51</v>
       </c>
       <c r="K12" t="s">
+        <v>88</v>
+      </c>
+      <c r="L12" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="L12" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="13" ht="14.25" spans="1:12">
       <c r="A13" t="s">
+        <v>90</v>
+      </c>
+      <c r="B13" t="s">
         <v>91</v>
-      </c>
-      <c r="B13" t="s">
-        <v>92</v>
       </c>
       <c r="C13" t="s">
         <v>38</v>
@@ -1790,7 +1784,7 @@
         <v>42</v>
       </c>
       <c r="I13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J13" t="s">
         <v>44</v>
@@ -1799,7 +1793,7 @@
         <v>66</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:12">

</xml_diff>

<commit_message>
feat: land MagicBook Step2 per-slot apply, formation ClassName/Lv, and BodyPart polish (v0.82.29)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="146">
   <si>
     <t>职业ID</t>
   </si>
@@ -259,6 +259,9 @@
     <t>Class_Warrior</t>
   </si>
   <si>
+    <t>战士2</t>
+  </si>
+  <si>
     <t>NormalAttackPrimaryMult_30|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|30_30|0.1_0.1</t>
   </si>
   <si>
@@ -271,16 +274,25 @@
     <t>Class_Archer</t>
   </si>
   <si>
+    <t>射手2</t>
+  </si>
+  <si>
     <t>App_0_11</t>
   </si>
   <si>
     <t>Class_Mage</t>
   </si>
   <si>
+    <t>法师2</t>
+  </si>
+  <si>
     <t>App_0_21</t>
   </si>
   <si>
     <t>Class_Rogue</t>
+  </si>
+  <si>
+    <t>盗贼2</t>
   </si>
   <si>
     <t>App_0_31</t>
@@ -1096,9 +1108,15 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1108,6 +1126,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1463,7 +1484,7 @@
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="3" max="3" width="9.5" customWidth="1"/>
-    <col min="4" max="4" width="15.5" customWidth="1"/>
+    <col min="4" max="4" width="15.5" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -1476,7 +1497,7 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
@@ -1523,7 +1544,7 @@
       <c r="C2" t="s">
         <v>17</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" t="s">
@@ -1570,7 +1591,7 @@
       <c r="C3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="3" t="s">
         <v>33</v>
       </c>
       <c r="E3" s="1" t="s">
@@ -1617,13 +1638,13 @@
       <c r="C4" t="s">
         <v>46</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <v>1</v>
       </c>
       <c r="E4" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>48</v>
       </c>
       <c r="G4">
@@ -1644,10 +1665,10 @@
       <c r="L4" t="s">
         <v>52</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="N4" s="4" t="s">
+      <c r="N4" s="6" t="s">
         <v>54</v>
       </c>
       <c r="O4" t="s">
@@ -1664,13 +1685,13 @@
       <c r="C5" t="s">
         <v>57</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="2">
         <v>1</v>
       </c>
       <c r="E5" t="s">
         <v>58</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="4" t="s">
         <v>59</v>
       </c>
       <c r="G5" t="s">
@@ -1691,10 +1712,10 @@
       <c r="L5" t="s">
         <v>61</v>
       </c>
-      <c r="M5" s="3">
+      <c r="M5" s="5">
         <v>4</v>
       </c>
-      <c r="N5" s="4" t="s">
+      <c r="N5" s="6" t="s">
         <v>62</v>
       </c>
       <c r="O5" t="s">
@@ -1711,13 +1732,13 @@
       <c r="C6" t="s">
         <v>65</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <v>1</v>
       </c>
       <c r="E6" t="s">
         <v>66</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="4" t="s">
         <v>59</v>
       </c>
       <c r="G6" t="s">
@@ -1738,10 +1759,10 @@
       <c r="L6" t="s">
         <v>61</v>
       </c>
-      <c r="M6" s="3">
+      <c r="M6" s="5">
         <v>3</v>
       </c>
-      <c r="N6" s="4" t="s">
+      <c r="N6" s="6" t="s">
         <v>69</v>
       </c>
       <c r="O6" t="s">
@@ -1758,13 +1779,13 @@
       <c r="C7" t="s">
         <v>71</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="2">
         <v>1</v>
       </c>
       <c r="E7" t="s">
         <v>58</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="4" t="s">
         <v>59</v>
       </c>
       <c r="G7">
@@ -1785,10 +1806,10 @@
       <c r="L7" t="s">
         <v>52</v>
       </c>
-      <c r="M7" s="3">
+      <c r="M7" s="5">
         <v>2</v>
       </c>
-      <c r="N7" s="4" t="s">
+      <c r="N7" s="6" t="s">
         <v>73</v>
       </c>
       <c r="O7" t="s">
@@ -1800,22 +1821,22 @@
         <v>74</v>
       </c>
       <c r="B8" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="C8" t="s">
         <v>46</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="2">
         <v>2</v>
       </c>
       <c r="E8" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>75</v>
+      <c r="F8" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="G8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H8" t="s">
         <v>49</v>
@@ -1832,11 +1853,11 @@
       <c r="L8" t="s">
         <v>52</v>
       </c>
-      <c r="M8" s="3" t="s">
+      <c r="M8" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="N8" s="4" t="s">
-        <v>77</v>
+      <c r="N8" s="6" t="s">
+        <v>78</v>
       </c>
       <c r="O8" t="s">
         <v>55</v>
@@ -1844,22 +1865,22 @@
     </row>
     <row r="9" ht="14.25" customHeight="1" spans="1:15">
       <c r="A9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
         <v>57</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="2">
         <v>2</v>
       </c>
       <c r="E9" t="s">
         <v>58</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>75</v>
+      <c r="F9" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="G9" t="s">
         <v>53</v>
@@ -1879,11 +1900,11 @@
       <c r="L9" t="s">
         <v>61</v>
       </c>
-      <c r="M9" s="3">
+      <c r="M9" s="5">
         <v>4</v>
       </c>
-      <c r="N9" s="4" t="s">
-        <v>79</v>
+      <c r="N9" s="6" t="s">
+        <v>81</v>
       </c>
       <c r="O9" t="s">
         <v>63</v>
@@ -1891,22 +1912,22 @@
     </row>
     <row r="10" ht="14.25" customHeight="1" spans="1:15">
       <c r="A10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B10" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="C10" t="s">
         <v>65</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="2">
         <v>2</v>
       </c>
       <c r="E10" t="s">
         <v>66</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>75</v>
+      <c r="F10" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="G10" t="s">
         <v>67</v>
@@ -1926,11 +1947,11 @@
       <c r="L10" t="s">
         <v>61</v>
       </c>
-      <c r="M10" s="3">
+      <c r="M10" s="5">
         <v>3</v>
       </c>
-      <c r="N10" s="4" t="s">
-        <v>81</v>
+      <c r="N10" s="6" t="s">
+        <v>84</v>
       </c>
       <c r="O10" t="s">
         <v>63</v>
@@ -1938,22 +1959,22 @@
     </row>
     <row r="11" ht="14.25" customHeight="1" spans="1:15">
       <c r="A11" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B11" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
         <v>71</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="2">
         <v>2</v>
       </c>
       <c r="E11" t="s">
         <v>58</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>75</v>
+      <c r="F11" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="G11">
         <v>0.35</v>
@@ -1973,11 +1994,11 @@
       <c r="L11" t="s">
         <v>52</v>
       </c>
-      <c r="M11" s="3">
+      <c r="M11" s="5">
         <v>2</v>
       </c>
-      <c r="N11" s="4" t="s">
-        <v>83</v>
+      <c r="N11" s="6" t="s">
+        <v>87</v>
       </c>
       <c r="O11" t="s">
         <v>63</v>
@@ -1985,22 +2006,22 @@
     </row>
     <row r="12" ht="14.25" customHeight="1" spans="1:15">
       <c r="A12" t="s">
-        <v>84</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>85</v>
+        <v>88</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>89</v>
       </c>
       <c r="C12" t="s">
         <v>46</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="2">
         <v>3</v>
       </c>
       <c r="E12" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>86</v>
+      <c r="F12" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="G12">
         <v>0.35</v>
@@ -2020,11 +2041,11 @@
       <c r="L12" t="s">
         <v>52</v>
       </c>
-      <c r="M12" s="3" t="s">
+      <c r="M12" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="N12" s="4" t="s">
-        <v>87</v>
+      <c r="N12" s="6" t="s">
+        <v>91</v>
       </c>
       <c r="O12" t="s">
         <v>63</v>
@@ -2032,22 +2053,22 @@
     </row>
     <row r="13" ht="14.25" customHeight="1" spans="1:15">
       <c r="A13" t="s">
-        <v>88</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>89</v>
+        <v>92</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>93</v>
       </c>
       <c r="C13" t="s">
         <v>57</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="2">
         <v>3</v>
       </c>
       <c r="E13" t="s">
         <v>58</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>86</v>
+      <c r="F13" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="G13" t="s">
         <v>53</v>
@@ -2067,11 +2088,11 @@
       <c r="L13" t="s">
         <v>61</v>
       </c>
-      <c r="M13" s="3">
+      <c r="M13" s="5">
         <v>4</v>
       </c>
-      <c r="N13" s="4" t="s">
-        <v>90</v>
+      <c r="N13" s="6" t="s">
+        <v>94</v>
       </c>
       <c r="O13" t="s">
         <v>63</v>
@@ -2079,22 +2100,22 @@
     </row>
     <row r="14" ht="14.25" customHeight="1" spans="1:15">
       <c r="A14" t="s">
-        <v>91</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>96</v>
       </c>
       <c r="C14" t="s">
         <v>65</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="2">
         <v>3</v>
       </c>
       <c r="E14" t="s">
         <v>66</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>86</v>
+      <c r="F14" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="G14" t="s">
         <v>67</v>
@@ -2114,11 +2135,11 @@
       <c r="L14" t="s">
         <v>61</v>
       </c>
-      <c r="M14" s="3">
+      <c r="M14" s="5">
         <v>3</v>
       </c>
-      <c r="N14" s="4" t="s">
-        <v>93</v>
+      <c r="N14" s="6" t="s">
+        <v>97</v>
       </c>
       <c r="O14" t="s">
         <v>63</v>
@@ -2126,22 +2147,22 @@
     </row>
     <row r="15" ht="14.25" customHeight="1" spans="1:15">
       <c r="A15" t="s">
-        <v>94</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>95</v>
+        <v>98</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>99</v>
       </c>
       <c r="C15" t="s">
         <v>71</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="2">
         <v>3</v>
       </c>
       <c r="E15" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>86</v>
+      <c r="F15" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="G15">
         <v>0.35</v>
@@ -2161,11 +2182,11 @@
       <c r="L15" t="s">
         <v>52</v>
       </c>
-      <c r="M15" s="3">
+      <c r="M15" s="5">
         <v>2</v>
       </c>
-      <c r="N15" s="4" t="s">
-        <v>96</v>
+      <c r="N15" s="6" t="s">
+        <v>100</v>
       </c>
       <c r="O15" t="s">
         <v>63</v>
@@ -2173,22 +2194,22 @@
     </row>
     <row r="16" ht="14.25" customHeight="1" spans="1:15">
       <c r="A16" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B16" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C16" t="s">
         <v>46</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="2">
         <v>3</v>
       </c>
       <c r="E16" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>86</v>
+      <c r="F16" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="G16">
         <v>0.35</v>
@@ -2208,11 +2229,11 @@
       <c r="L16" t="s">
         <v>52</v>
       </c>
-      <c r="M16" s="3" t="s">
+      <c r="M16" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="N16" s="4" t="s">
-        <v>99</v>
+      <c r="N16" s="6" t="s">
+        <v>103</v>
       </c>
       <c r="O16" t="s">
         <v>63</v>
@@ -2220,22 +2241,22 @@
     </row>
     <row r="17" ht="14.25" customHeight="1" spans="1:15">
       <c r="A17" t="s">
-        <v>100</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>101</v>
+        <v>104</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>105</v>
       </c>
       <c r="C17" t="s">
         <v>57</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="2">
         <v>3</v>
       </c>
       <c r="E17" t="s">
         <v>58</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>86</v>
+      <c r="F17" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="G17" t="s">
         <v>53</v>
@@ -2255,11 +2276,11 @@
       <c r="L17" t="s">
         <v>61</v>
       </c>
-      <c r="M17" s="3">
+      <c r="M17" s="5">
         <v>4</v>
       </c>
-      <c r="N17" s="4" t="s">
-        <v>102</v>
+      <c r="N17" s="6" t="s">
+        <v>106</v>
       </c>
       <c r="O17" t="s">
         <v>63</v>
@@ -2267,22 +2288,22 @@
     </row>
     <row r="18" ht="14.25" customHeight="1" spans="1:15">
       <c r="A18" t="s">
-        <v>103</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>108</v>
       </c>
       <c r="C18" t="s">
         <v>65</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="2">
         <v>3</v>
       </c>
       <c r="E18" t="s">
         <v>66</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>86</v>
+      <c r="F18" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="G18" t="s">
         <v>67</v>
@@ -2302,11 +2323,11 @@
       <c r="L18" t="s">
         <v>61</v>
       </c>
-      <c r="M18" s="3">
+      <c r="M18" s="5">
         <v>3</v>
       </c>
-      <c r="N18" s="4" t="s">
-        <v>105</v>
+      <c r="N18" s="6" t="s">
+        <v>109</v>
       </c>
       <c r="O18" t="s">
         <v>63</v>
@@ -2314,22 +2335,22 @@
     </row>
     <row r="19" ht="14.25" customHeight="1" spans="1:15">
       <c r="A19" t="s">
-        <v>106</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>107</v>
+        <v>110</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>111</v>
       </c>
       <c r="C19" t="s">
         <v>71</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="2">
         <v>3</v>
       </c>
       <c r="E19" t="s">
         <v>66</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>86</v>
+      <c r="F19" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="G19">
         <v>0.35</v>
@@ -2349,11 +2370,11 @@
       <c r="L19" t="s">
         <v>52</v>
       </c>
-      <c r="M19" s="3">
+      <c r="M19" s="5">
         <v>2</v>
       </c>
-      <c r="N19" s="4" t="s">
-        <v>108</v>
+      <c r="N19" s="6" t="s">
+        <v>112</v>
       </c>
       <c r="O19" t="s">
         <v>63</v>
@@ -2361,22 +2382,22 @@
     </row>
     <row r="20" spans="1:15">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B20" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C20" t="s">
         <v>46</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="2">
         <v>4</v>
       </c>
       <c r="E20" t="s">
         <v>47</v>
       </c>
-      <c r="F20" s="2" t="s">
-        <v>111</v>
+      <c r="F20" s="4" t="s">
+        <v>115</v>
       </c>
       <c r="G20" t="s">
         <v>49</v>
@@ -2391,16 +2412,16 @@
         <v>50</v>
       </c>
       <c r="K20" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="L20" t="s">
         <v>52</v>
       </c>
-      <c r="M20" s="3">
+      <c r="M20" s="5">
         <v>1</v>
       </c>
-      <c r="N20" s="5" t="s">
-        <v>113</v>
+      <c r="N20" s="7" t="s">
+        <v>117</v>
       </c>
       <c r="O20" t="s">
         <v>63</v>
@@ -2408,22 +2429,22 @@
     </row>
     <row r="21" ht="14.25" customHeight="1" spans="1:15">
       <c r="A21" t="s">
-        <v>114</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>119</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="2">
         <v>4</v>
       </c>
       <c r="E21" t="s">
         <v>66</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>111</v>
+      <c r="F21" s="4" t="s">
+        <v>115</v>
       </c>
       <c r="G21" t="s">
         <v>67</v>
@@ -2443,245 +2464,245 @@
       <c r="L21" t="s">
         <v>61</v>
       </c>
-      <c r="M21" s="3">
+      <c r="M21" s="5">
         <v>2</v>
       </c>
-      <c r="N21" s="5" t="s">
-        <v>116</v>
+      <c r="N21" s="7" t="s">
+        <v>120</v>
       </c>
       <c r="O21" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1" spans="1:15">
-      <c r="A22" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>118</v>
+      <c r="A22" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>122</v>
       </c>
       <c r="C22" t="s">
         <v>46</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="9">
         <v>1</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="G22" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="I22" s="6" t="s">
+      <c r="G22" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I22" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="J22" s="6" t="s">
+      <c r="J22" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="K22" s="6" t="s">
+      <c r="K22" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="L22" s="6" t="s">
+      <c r="L22" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="M22" s="7" t="s">
+      <c r="M22" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="N22" s="8" t="s">
-        <v>119</v>
+      <c r="N22" s="11" t="s">
+        <v>123</v>
       </c>
       <c r="O22" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1" spans="1:15">
-      <c r="A23" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>121</v>
+      <c r="A23" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>125</v>
       </c>
       <c r="C23" t="s">
         <v>65</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="9">
         <v>1</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F23" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="G23" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="H23" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="I23" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J23" s="6" t="s">
+      <c r="G23" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="J23" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="K23" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="L23" s="6" t="s">
+      <c r="K23" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="L23" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="M23" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="N23" s="8" t="s">
-        <v>125</v>
+      <c r="M23" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="N23" s="11" t="s">
+        <v>129</v>
       </c>
       <c r="O23" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1" spans="1:15">
-      <c r="A24" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>127</v>
+      <c r="A24" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>131</v>
       </c>
       <c r="C24" t="s">
         <v>57</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="9">
         <v>1</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="F24" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="G24" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="J24" s="6" t="s">
+      <c r="G24" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="J24" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="K24" s="6" t="s">
+      <c r="K24" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="L24" s="6" t="s">
+      <c r="L24" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="M24" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="N24" s="8" t="s">
-        <v>131</v>
+      <c r="M24" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="N24" s="11" t="s">
+        <v>135</v>
       </c>
       <c r="O24" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="25" ht="14.25" customHeight="1" spans="1:15">
-      <c r="A25" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>133</v>
+      <c r="A25" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>137</v>
       </c>
       <c r="C25" t="s">
         <v>65</v>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="9">
         <v>1</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="E25" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="F25" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="G25" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="H25" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="J25" s="6" t="s">
+      <c r="G25" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="J25" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="K25" s="6" t="s">
+      <c r="K25" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="L25" s="6" t="s">
+      <c r="L25" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="M25" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="N25" s="8" t="s">
-        <v>137</v>
+      <c r="M25" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="N25" s="11" t="s">
+        <v>141</v>
       </c>
       <c r="O25" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:15">
-      <c r="A26" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>139</v>
+      <c r="A26" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>143</v>
       </c>
       <c r="C26" t="s">
         <v>46</v>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="9">
         <v>1</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="E26" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="F26" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="G26" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="I26" s="6" t="s">
+      <c r="G26" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="H26" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I26" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="J26" s="6" t="s">
+      <c r="J26" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="K26" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="L26" s="6" t="s">
+      <c r="K26" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="L26" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="M26" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="N26" s="6" t="s">
+      <c r="M26" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="N26" s="8" t="s">
         <v>63</v>
       </c>
       <c r="O26" t="s">

</xml_diff>

<commit_message>
feat: land CombatConstantConfig, FormationClassZones sync, and MetaShell label polish (v0.82.34)
EOF

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Work\Cursor\Gravedigger2026\Gravedigger2026\Gravedigger2026\Assets\ConfigTables\Mode2\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\CursorGame_Git\Gravedigger2026\Gravedigger2026\Assets\ConfigTables\Mode2\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255"/>
+    <workbookView windowWidth="25600" windowHeight="12080"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="121">
   <si>
     <t>职业ID</t>
   </si>
@@ -395,81 +395,6 @@
   </si>
   <si>
     <t>App_5_51</t>
-  </si>
-  <si>
-    <t>Class_Knight</t>
-  </si>
-  <si>
-    <t>骑士</t>
-  </si>
-  <si>
-    <t>App_05</t>
-  </si>
-  <si>
-    <t>Class_Priest</t>
-  </si>
-  <si>
-    <t>牧师</t>
-  </si>
-  <si>
-    <t>1.2</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>App_09</t>
-  </si>
-  <si>
-    <t>Class_Ranger</t>
-  </si>
-  <si>
-    <t>游侠</t>
-  </si>
-  <si>
-    <t>1.1</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>App_03</t>
-  </si>
-  <si>
-    <t>Class_Warlock</t>
-  </si>
-  <si>
-    <t>术士</t>
-  </si>
-  <si>
-    <t>0.9</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>App_08</t>
-  </si>
-  <si>
-    <t>Class_Servants</t>
-  </si>
-  <si>
-    <t>仆从</t>
-  </si>
-  <si>
-    <t>2.5</t>
-  </si>
-  <si>
-    <t>11</t>
   </si>
 </sst>
 </file>
@@ -642,7 +567,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -658,12 +583,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -984,7 +903,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
@@ -1008,16 +927,16 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="6">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="6">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="7">
@@ -1026,89 +945,89 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="13" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="35" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1125,14 +1044,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1479,12 +1390,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:O26"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <dimension ref="A1:O21"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="3" max="3" width="9.5" customWidth="1"/>
     <col min="4" max="4" width="15.5" style="2" customWidth="1"/>
+    <col min="6" max="6" width="30.6363636363636" customWidth="1"/>
+    <col min="7" max="7" width="21.5454545454545" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -2471,241 +2384,6 @@
         <v>120</v>
       </c>
       <c r="O21" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="22" ht="14.25" customHeight="1" spans="1:15">
-      <c r="A22" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="C22" t="s">
-        <v>46</v>
-      </c>
-      <c r="D22" s="9">
-        <v>1</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="I22" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="J22" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="K22" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="L22" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="M22" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="N22" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="O22" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="23" ht="14.25" customHeight="1" spans="1:15">
-      <c r="A23" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="C23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D23" s="9">
-        <v>1</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="G23" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="H23" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="J23" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="K23" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="L23" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="M23" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="N23" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="O23" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="24" ht="14.25" customHeight="1" spans="1:15">
-      <c r="A24" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="C24" t="s">
-        <v>57</v>
-      </c>
-      <c r="D24" s="9">
-        <v>1</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="F24" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="G24" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="H24" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="I24" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="J24" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="K24" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="L24" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="M24" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="N24" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="O24" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="25" ht="14.25" customHeight="1" spans="1:15">
-      <c r="A25" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="C25" t="s">
-        <v>65</v>
-      </c>
-      <c r="D25" s="9">
-        <v>1</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="H25" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="I25" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="J25" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="K25" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="L25" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="M25" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="N25" s="11" t="s">
-        <v>141</v>
-      </c>
-      <c r="O25" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15">
-      <c r="A26" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="C26" t="s">
-        <v>46</v>
-      </c>
-      <c r="D26" s="9">
-        <v>1</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="H26" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="J26" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="K26" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="L26" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="M26" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="N26" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="O26" t="s">
         <v>63</v>
       </c>
     </row>

</xml_diff>